<commit_message>
anaylsis of 2016 turning point
</commit_message>
<xml_diff>
--- a/reports/country_participation_trend/country_participation_analysis.xlsx
+++ b/reports/country_participation_trend/country_participation_analysis.xlsx
@@ -1318,13 +1318,13 @@
         <v>3020</v>
       </c>
       <c r="C28" t="n">
-        <v>2934</v>
+        <v>2933</v>
       </c>
       <c r="D28" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E28" t="n">
-        <v>0.02847682119205298</v>
+        <v>0.02880794701986755</v>
       </c>
       <c r="F28" t="n">
         <v>103</v>
@@ -1346,16 +1346,16 @@
         <v>2018</v>
       </c>
       <c r="B29" t="n">
-        <v>3170</v>
+        <v>3171</v>
       </c>
       <c r="C29" t="n">
-        <v>3103</v>
+        <v>3104</v>
       </c>
       <c r="D29" t="n">
         <v>67</v>
       </c>
       <c r="E29" t="n">
-        <v>0.02113564668769716</v>
+        <v>0.02112898139388206</v>
       </c>
       <c r="F29" t="n">
         <v>108</v>
@@ -1408,16 +1408,16 @@
         <v>2020</v>
       </c>
       <c r="B31" t="n">
-        <v>3337</v>
+        <v>3338</v>
       </c>
       <c r="C31" t="n">
-        <v>3203</v>
+        <v>3204</v>
       </c>
       <c r="D31" t="n">
         <v>134</v>
       </c>
       <c r="E31" t="n">
-        <v>0.04015582858855259</v>
+        <v>0.04014379868184541</v>
       </c>
       <c r="F31" t="n">
         <v>91</v>
@@ -1439,16 +1439,16 @@
         <v>2021</v>
       </c>
       <c r="B32" t="n">
-        <v>4079</v>
+        <v>4081</v>
       </c>
       <c r="C32" t="n">
-        <v>3926</v>
+        <v>3928</v>
       </c>
       <c r="D32" t="n">
         <v>153</v>
       </c>
       <c r="E32" t="n">
-        <v>0.03750919342976219</v>
+        <v>0.03749081107571674</v>
       </c>
       <c r="F32" t="n">
         <v>102</v>
@@ -1501,16 +1501,16 @@
         <v>2023</v>
       </c>
       <c r="B34" t="n">
-        <v>3583</v>
+        <v>3584</v>
       </c>
       <c r="C34" t="n">
-        <v>3435</v>
+        <v>3437</v>
       </c>
       <c r="D34" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="E34" t="n">
-        <v>0.04130616801562936</v>
+        <v>0.041015625</v>
       </c>
       <c r="F34" t="n">
         <v>94</v>
@@ -1566,13 +1566,13 @@
         <v>3784</v>
       </c>
       <c r="C36" t="n">
-        <v>3521</v>
+        <v>3526</v>
       </c>
       <c r="D36" t="n">
-        <v>263</v>
+        <v>258</v>
       </c>
       <c r="E36" t="n">
-        <v>0.06950317124735729</v>
+        <v>0.06818181818181818</v>
       </c>
       <c r="F36" t="n">
         <v>85</v>
@@ -1594,16 +1594,16 @@
         <v>2026</v>
       </c>
       <c r="B37" t="n">
-        <v>2717</v>
+        <v>2827</v>
       </c>
       <c r="C37" t="n">
-        <v>2196</v>
+        <v>2301</v>
       </c>
       <c r="D37" t="n">
-        <v>521</v>
+        <v>526</v>
       </c>
       <c r="E37" t="n">
-        <v>0.1917556128082444</v>
+        <v>0.186062964273081</v>
       </c>
       <c r="F37" t="n">
         <v>74</v>
@@ -1755,7 +1755,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>/Users/mac/Desktop/pfizerProj/nexus-permissible-analysis/runs/run_20260722T020135Z</t>
+          <t>/Users/mac/Desktop/pfizerProj/nexus-permissible-analysis/runs/run_20260730T061844Z</t>
         </is>
       </c>
     </row>
@@ -1767,7 +1767,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-30</t>
         </is>
       </c>
     </row>
@@ -2574,7 +2574,7 @@
         <v>3020</v>
       </c>
       <c r="C28" t="n">
-        <v>2934</v>
+        <v>2933</v>
       </c>
       <c r="D28" t="n">
         <v>70</v>
@@ -2583,7 +2583,7 @@
         <v>0.02317880794701987</v>
       </c>
       <c r="F28" t="n">
-        <v>0.02385821404226312</v>
+        <v>0.02386634844868735</v>
       </c>
       <c r="G28" t="n">
         <v>49.33333333333334</v>
@@ -2599,19 +2599,19 @@
         <v>2018</v>
       </c>
       <c r="B29" t="n">
-        <v>3170</v>
+        <v>3171</v>
       </c>
       <c r="C29" t="n">
-        <v>3103</v>
+        <v>3104</v>
       </c>
       <c r="D29" t="n">
         <v>106</v>
       </c>
       <c r="E29" t="n">
-        <v>0.03343848580441641</v>
+        <v>0.03342794071270892</v>
       </c>
       <c r="F29" t="n">
-        <v>0.03416048984853368</v>
+        <v>0.03414948453608247</v>
       </c>
       <c r="G29" t="n">
         <v>71</v>
@@ -2655,19 +2655,19 @@
         <v>2020</v>
       </c>
       <c r="B31" t="n">
-        <v>3337</v>
+        <v>3338</v>
       </c>
       <c r="C31" t="n">
-        <v>3203</v>
+        <v>3204</v>
       </c>
       <c r="D31" t="n">
         <v>148</v>
       </c>
       <c r="E31" t="n">
-        <v>0.04435121366496853</v>
+        <v>0.04433792690233673</v>
       </c>
       <c r="F31" t="n">
-        <v>0.04620668123634093</v>
+        <v>0.04619225967540574</v>
       </c>
       <c r="G31" t="n">
         <v>129</v>
@@ -2683,22 +2683,22 @@
         <v>2021</v>
       </c>
       <c r="B32" t="n">
-        <v>4079</v>
+        <v>4081</v>
       </c>
       <c r="C32" t="n">
-        <v>3926</v>
+        <v>3928</v>
       </c>
       <c r="D32" t="n">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="E32" t="n">
-        <v>0.05123804854130914</v>
+        <v>0.0509679000245038</v>
       </c>
       <c r="F32" t="n">
-        <v>0.0532348446255731</v>
+        <v>0.05295315682281059</v>
       </c>
       <c r="G32" t="n">
-        <v>163.3333333333333</v>
+        <v>163</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -2726,7 +2726,7 @@
         <v>0.05614823133071308</v>
       </c>
       <c r="G33" t="n">
-        <v>185.6666666666667</v>
+        <v>185.3333333333333</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -2739,19 +2739,19 @@
         <v>2023</v>
       </c>
       <c r="B34" t="n">
-        <v>3583</v>
+        <v>3584</v>
       </c>
       <c r="C34" t="n">
-        <v>3435</v>
+        <v>3437</v>
       </c>
       <c r="D34" t="n">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="E34" t="n">
-        <v>0.05888919899525537</v>
+        <v>0.05915178571428571</v>
       </c>
       <c r="F34" t="n">
-        <v>0.06142649199417758</v>
+        <v>0.06168169915624091</v>
       </c>
       <c r="G34" t="n">
         <v>206.6666666666667</v>
@@ -2773,13 +2773,13 @@
         <v>3379</v>
       </c>
       <c r="D35" t="n">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="E35" t="n">
-        <v>0.05763850027979855</v>
+        <v>0.05735870173475098</v>
       </c>
       <c r="F35" t="n">
-        <v>0.06096478248002368</v>
+        <v>0.06066883693400414</v>
       </c>
       <c r="G35" t="n">
         <v>205.6666666666667</v>
@@ -2798,19 +2798,19 @@
         <v>3784</v>
       </c>
       <c r="C36" t="n">
-        <v>3521</v>
+        <v>3526</v>
       </c>
       <c r="D36" t="n">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="E36" t="n">
-        <v>0.07716701902748414</v>
+        <v>0.07769556025369979</v>
       </c>
       <c r="F36" t="n">
-        <v>0.08293098551547856</v>
+        <v>0.08338060124787294</v>
       </c>
       <c r="G36" t="n">
-        <v>236.3333333333333</v>
+        <v>237</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -2823,22 +2823,22 @@
         <v>2026</v>
       </c>
       <c r="B37" t="n">
-        <v>2717</v>
+        <v>2827</v>
       </c>
       <c r="C37" t="n">
-        <v>2196</v>
+        <v>2301</v>
       </c>
       <c r="D37" t="n">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="E37" t="n">
-        <v>0.03827751196172249</v>
+        <v>0.03855677396533427</v>
       </c>
       <c r="F37" t="n">
-        <v>0.04735883424408015</v>
+        <v>0.04737070838765754</v>
       </c>
       <c r="G37" t="n">
-        <v>200.6666666666667</v>
+        <v>202.6666666666667</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -15564,10 +15564,10 @@
         <v>0.03178807947019868</v>
       </c>
       <c r="F158" t="n">
-        <v>2934</v>
+        <v>2933</v>
       </c>
       <c r="G158" t="n">
-        <v>0.032719836400818</v>
+        <v>0.03273099215819979</v>
       </c>
       <c r="H158" t="inlineStr">
         <is>
@@ -15588,16 +15588,16 @@
         <v>3020</v>
       </c>
       <c r="D159" t="n">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="E159" t="n">
-        <v>0.3519867549668874</v>
+        <v>0.3516556291390728</v>
       </c>
       <c r="F159" t="n">
-        <v>2934</v>
+        <v>2933</v>
       </c>
       <c r="G159" t="n">
-        <v>0.3623040218132242</v>
+        <v>0.3620866007500853</v>
       </c>
       <c r="H159" t="inlineStr">
         <is>
@@ -15618,16 +15618,16 @@
         <v>3020</v>
       </c>
       <c r="D160" t="n">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="E160" t="n">
-        <v>0.4182119205298013</v>
+        <v>0.4178807947019867</v>
       </c>
       <c r="F160" t="n">
-        <v>2934</v>
+        <v>2933</v>
       </c>
       <c r="G160" t="n">
-        <v>0.4304703476482618</v>
+        <v>0.4302761677463348</v>
       </c>
       <c r="H160" t="inlineStr">
         <is>
@@ -15648,16 +15648,16 @@
         <v>3020</v>
       </c>
       <c r="D161" t="n">
-        <v>1701</v>
+        <v>1700</v>
       </c>
       <c r="E161" t="n">
-        <v>0.5632450331125828</v>
+        <v>0.5629139072847682</v>
       </c>
       <c r="F161" t="n">
-        <v>2934</v>
+        <v>2933</v>
       </c>
       <c r="G161" t="n">
-        <v>0.5797546012269938</v>
+        <v>0.5796113194681214</v>
       </c>
       <c r="H161" t="inlineStr">
         <is>
@@ -15678,16 +15678,16 @@
         <v>3020</v>
       </c>
       <c r="D162" t="n">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="E162" t="n">
-        <v>0.06622516556291391</v>
+        <v>0.06589403973509934</v>
       </c>
       <c r="F162" t="n">
-        <v>2934</v>
+        <v>2933</v>
       </c>
       <c r="G162" t="n">
-        <v>0.0681663258350375</v>
+        <v>0.06784861916126833</v>
       </c>
       <c r="H162" t="inlineStr">
         <is>
@@ -15708,16 +15708,16 @@
         <v>3020</v>
       </c>
       <c r="D163" t="n">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="E163" t="n">
-        <v>0.1182119205298013</v>
+        <v>0.1178807947019868</v>
       </c>
       <c r="F163" t="n">
-        <v>2934</v>
+        <v>2933</v>
       </c>
       <c r="G163" t="n">
-        <v>0.1216768916155419</v>
+        <v>0.1213774292533242</v>
       </c>
       <c r="H163" t="inlineStr">
         <is>
@@ -15735,19 +15735,19 @@
         </is>
       </c>
       <c r="C164" t="n">
-        <v>3170</v>
+        <v>3171</v>
       </c>
       <c r="D164" t="n">
         <v>107</v>
       </c>
       <c r="E164" t="n">
-        <v>0.03375394321766562</v>
+        <v>0.0337432986439609</v>
       </c>
       <c r="F164" t="n">
-        <v>3103</v>
+        <v>3104</v>
       </c>
       <c r="G164" t="n">
-        <v>0.03448275862068965</v>
+        <v>0.03447164948453608</v>
       </c>
       <c r="H164" t="inlineStr">
         <is>
@@ -15765,19 +15765,19 @@
         </is>
       </c>
       <c r="C165" t="n">
-        <v>3170</v>
+        <v>3171</v>
       </c>
       <c r="D165" t="n">
         <v>1181</v>
       </c>
       <c r="E165" t="n">
-        <v>0.3725552050473186</v>
+        <v>0.3724377168085777</v>
       </c>
       <c r="F165" t="n">
-        <v>3103</v>
+        <v>3104</v>
       </c>
       <c r="G165" t="n">
-        <v>0.3805994199162101</v>
+        <v>0.3804768041237113</v>
       </c>
       <c r="H165" t="inlineStr">
         <is>
@@ -15795,19 +15795,19 @@
         </is>
       </c>
       <c r="C166" t="n">
-        <v>3170</v>
+        <v>3171</v>
       </c>
       <c r="D166" t="n">
-        <v>1255</v>
+        <v>1256</v>
       </c>
       <c r="E166" t="n">
-        <v>0.3958990536277602</v>
+        <v>0.3960895616524756</v>
       </c>
       <c r="F166" t="n">
-        <v>3103</v>
+        <v>3104</v>
       </c>
       <c r="G166" t="n">
-        <v>0.4044473090557525</v>
+        <v>0.404639175257732</v>
       </c>
       <c r="H166" t="inlineStr">
         <is>
@@ -15825,19 +15825,19 @@
         </is>
       </c>
       <c r="C167" t="n">
-        <v>3170</v>
+        <v>3171</v>
       </c>
       <c r="D167" t="n">
         <v>1811</v>
       </c>
       <c r="E167" t="n">
-        <v>0.5712933753943218</v>
+        <v>0.5711132134973195</v>
       </c>
       <c r="F167" t="n">
-        <v>3103</v>
+        <v>3104</v>
       </c>
       <c r="G167" t="n">
-        <v>0.5836287463744763</v>
+        <v>0.5834407216494846</v>
       </c>
       <c r="H167" t="inlineStr">
         <is>
@@ -15855,19 +15855,19 @@
         </is>
       </c>
       <c r="C168" t="n">
-        <v>3170</v>
+        <v>3171</v>
       </c>
       <c r="D168" t="n">
         <v>234</v>
       </c>
       <c r="E168" t="n">
-        <v>0.07381703470031546</v>
+        <v>0.07379375591296121</v>
       </c>
       <c r="F168" t="n">
-        <v>3103</v>
+        <v>3104</v>
       </c>
       <c r="G168" t="n">
-        <v>0.07541089268449887</v>
+        <v>0.07538659793814433</v>
       </c>
       <c r="H168" t="inlineStr">
         <is>
@@ -15885,19 +15885,19 @@
         </is>
       </c>
       <c r="C169" t="n">
-        <v>3170</v>
+        <v>3171</v>
       </c>
       <c r="D169" t="n">
         <v>394</v>
       </c>
       <c r="E169" t="n">
-        <v>0.1242902208201893</v>
+        <v>0.1242510249132766</v>
       </c>
       <c r="F169" t="n">
-        <v>3103</v>
+        <v>3104</v>
       </c>
       <c r="G169" t="n">
-        <v>0.1269738962294554</v>
+        <v>0.1269329896907216</v>
       </c>
       <c r="H169" t="inlineStr">
         <is>
@@ -16095,19 +16095,19 @@
         </is>
       </c>
       <c r="C176" t="n">
-        <v>3337</v>
+        <v>3338</v>
       </c>
       <c r="D176" t="n">
         <v>88</v>
       </c>
       <c r="E176" t="n">
-        <v>0.02637099190890021</v>
+        <v>0.02636309167165968</v>
       </c>
       <c r="F176" t="n">
-        <v>3203</v>
+        <v>3204</v>
       </c>
       <c r="G176" t="n">
-        <v>0.0274742428972838</v>
+        <v>0.02746566791510612</v>
       </c>
       <c r="H176" t="inlineStr">
         <is>
@@ -16125,19 +16125,19 @@
         </is>
       </c>
       <c r="C177" t="n">
-        <v>3337</v>
+        <v>3338</v>
       </c>
       <c r="D177" t="n">
         <v>1438</v>
       </c>
       <c r="E177" t="n">
-        <v>0.4309259814204375</v>
+        <v>0.4307968843618933</v>
       </c>
       <c r="F177" t="n">
-        <v>3203</v>
+        <v>3204</v>
       </c>
       <c r="G177" t="n">
-        <v>0.4489541055260693</v>
+        <v>0.4488139825218477</v>
       </c>
       <c r="H177" t="inlineStr">
         <is>
@@ -16155,19 +16155,19 @@
         </is>
       </c>
       <c r="C178" t="n">
-        <v>3337</v>
+        <v>3338</v>
       </c>
       <c r="D178" t="n">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="E178" t="n">
-        <v>0.3545100389571471</v>
+        <v>0.3547034152186938</v>
       </c>
       <c r="F178" t="n">
-        <v>3203</v>
+        <v>3204</v>
       </c>
       <c r="G178" t="n">
-        <v>0.3693412425850765</v>
+        <v>0.369538077403246</v>
       </c>
       <c r="H178" t="inlineStr">
         <is>
@@ -16185,19 +16185,19 @@
         </is>
       </c>
       <c r="C179" t="n">
-        <v>3337</v>
+        <v>3338</v>
       </c>
       <c r="D179" t="n">
         <v>1752</v>
       </c>
       <c r="E179" t="n">
-        <v>0.525022475277195</v>
+        <v>0.5248651887357699</v>
       </c>
       <c r="F179" t="n">
-        <v>3203</v>
+        <v>3204</v>
       </c>
       <c r="G179" t="n">
-        <v>0.5469871995004683</v>
+        <v>0.5468164794007491</v>
       </c>
       <c r="H179" t="inlineStr">
         <is>
@@ -16215,19 +16215,19 @@
         </is>
       </c>
       <c r="C180" t="n">
-        <v>3337</v>
+        <v>3338</v>
       </c>
       <c r="D180" t="n">
         <v>297</v>
       </c>
       <c r="E180" t="n">
-        <v>0.08900209769253821</v>
+        <v>0.0889754343918514</v>
       </c>
       <c r="F180" t="n">
-        <v>3203</v>
+        <v>3204</v>
       </c>
       <c r="G180" t="n">
-        <v>0.09272556977833281</v>
+        <v>0.09269662921348315</v>
       </c>
       <c r="H180" t="inlineStr">
         <is>
@@ -16245,19 +16245,19 @@
         </is>
       </c>
       <c r="C181" t="n">
-        <v>3337</v>
+        <v>3338</v>
       </c>
       <c r="D181" t="n">
         <v>454</v>
       </c>
       <c r="E181" t="n">
-        <v>0.136050344620917</v>
+        <v>0.1360095865787897</v>
       </c>
       <c r="F181" t="n">
-        <v>3203</v>
+        <v>3204</v>
       </c>
       <c r="G181" t="n">
-        <v>0.1417421167655323</v>
+        <v>0.1416978776529338</v>
       </c>
       <c r="H181" t="inlineStr">
         <is>
@@ -16275,19 +16275,19 @@
         </is>
       </c>
       <c r="C182" t="n">
-        <v>4079</v>
+        <v>4081</v>
       </c>
       <c r="D182" t="n">
         <v>121</v>
       </c>
       <c r="E182" t="n">
-        <v>0.02966413336602108</v>
+        <v>0.02964959568733154</v>
       </c>
       <c r="F182" t="n">
-        <v>3926</v>
+        <v>3928</v>
       </c>
       <c r="G182" t="n">
-        <v>0.03082017320427917</v>
+        <v>0.03080448065173116</v>
       </c>
       <c r="H182" t="inlineStr">
         <is>
@@ -16305,19 +16305,19 @@
         </is>
       </c>
       <c r="C183" t="n">
-        <v>4079</v>
+        <v>4081</v>
       </c>
       <c r="D183" t="n">
-        <v>1884</v>
+        <v>1885</v>
       </c>
       <c r="E183" t="n">
-        <v>0.461877911252758</v>
+        <v>0.4618965939720657</v>
       </c>
       <c r="F183" t="n">
-        <v>3926</v>
+        <v>3928</v>
       </c>
       <c r="G183" t="n">
-        <v>0.4798777381558839</v>
+        <v>0.479887983706721</v>
       </c>
       <c r="H183" t="inlineStr">
         <is>
@@ -16335,19 +16335,19 @@
         </is>
       </c>
       <c r="C184" t="n">
-        <v>4079</v>
+        <v>4081</v>
       </c>
       <c r="D184" t="n">
         <v>1398</v>
       </c>
       <c r="E184" t="n">
-        <v>0.3427310615346899</v>
+        <v>0.3425630972800784</v>
       </c>
       <c r="F184" t="n">
-        <v>3926</v>
+        <v>3928</v>
       </c>
       <c r="G184" t="n">
-        <v>0.3560876209882832</v>
+        <v>0.3559063136456212</v>
       </c>
       <c r="H184" t="inlineStr">
         <is>
@@ -16365,19 +16365,19 @@
         </is>
       </c>
       <c r="C185" t="n">
-        <v>4079</v>
+        <v>4081</v>
       </c>
       <c r="D185" t="n">
         <v>2087</v>
       </c>
       <c r="E185" t="n">
-        <v>0.5116450110321157</v>
+        <v>0.5113942661112473</v>
       </c>
       <c r="F185" t="n">
-        <v>3926</v>
+        <v>3928</v>
       </c>
       <c r="G185" t="n">
-        <v>0.5315843097300051</v>
+        <v>0.5313136456211812</v>
       </c>
       <c r="H185" t="inlineStr">
         <is>
@@ -16395,19 +16395,19 @@
         </is>
       </c>
       <c r="C186" t="n">
-        <v>4079</v>
+        <v>4081</v>
       </c>
       <c r="D186" t="n">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="E186" t="n">
-        <v>0.07697965187545967</v>
+        <v>0.07669688801764274</v>
       </c>
       <c r="F186" t="n">
-        <v>3926</v>
+        <v>3928</v>
       </c>
       <c r="G186" t="n">
-        <v>0.07997962302598065</v>
+        <v>0.07968431771894094</v>
       </c>
       <c r="H186" t="inlineStr">
         <is>
@@ -16425,19 +16425,19 @@
         </is>
       </c>
       <c r="C187" t="n">
-        <v>4079</v>
+        <v>4081</v>
       </c>
       <c r="D187" t="n">
         <v>540</v>
       </c>
       <c r="E187" t="n">
-        <v>0.1323853885756313</v>
+        <v>0.1323205096790002</v>
       </c>
       <c r="F187" t="n">
-        <v>3926</v>
+        <v>3928</v>
       </c>
       <c r="G187" t="n">
-        <v>0.1375445746306674</v>
+        <v>0.1374745417515275</v>
       </c>
       <c r="H187" t="inlineStr">
         <is>
@@ -16635,19 +16635,19 @@
         </is>
       </c>
       <c r="C194" t="n">
-        <v>3583</v>
+        <v>3584</v>
       </c>
       <c r="D194" t="n">
         <v>108</v>
       </c>
       <c r="E194" t="n">
-        <v>0.03014233882221602</v>
+        <v>0.03013392857142857</v>
       </c>
       <c r="F194" t="n">
-        <v>3435</v>
+        <v>3437</v>
       </c>
       <c r="G194" t="n">
-        <v>0.0314410480349345</v>
+        <v>0.03142275240034914</v>
       </c>
       <c r="H194" t="inlineStr">
         <is>
@@ -16665,19 +16665,19 @@
         </is>
       </c>
       <c r="C195" t="n">
-        <v>3583</v>
+        <v>3584</v>
       </c>
       <c r="D195" t="n">
-        <v>1818</v>
+        <v>1820</v>
       </c>
       <c r="E195" t="n">
-        <v>0.5073960368406364</v>
+        <v>0.5078125</v>
       </c>
       <c r="F195" t="n">
-        <v>3435</v>
+        <v>3437</v>
       </c>
       <c r="G195" t="n">
-        <v>0.5292576419213973</v>
+        <v>0.5295315682281059</v>
       </c>
       <c r="H195" t="inlineStr">
         <is>
@@ -16695,19 +16695,19 @@
         </is>
       </c>
       <c r="C196" t="n">
-        <v>3583</v>
+        <v>3584</v>
       </c>
       <c r="D196" t="n">
         <v>1071</v>
       </c>
       <c r="E196" t="n">
-        <v>0.2989115266536422</v>
+        <v>0.298828125</v>
       </c>
       <c r="F196" t="n">
-        <v>3435</v>
+        <v>3437</v>
       </c>
       <c r="G196" t="n">
-        <v>0.3117903930131005</v>
+        <v>0.3116089613034623</v>
       </c>
       <c r="H196" t="inlineStr">
         <is>
@@ -16725,19 +16725,19 @@
         </is>
       </c>
       <c r="C197" t="n">
-        <v>3583</v>
+        <v>3584</v>
       </c>
       <c r="D197" t="n">
-        <v>1676</v>
+        <v>1677</v>
       </c>
       <c r="E197" t="n">
-        <v>0.467764443204019</v>
+        <v>0.4679129464285715</v>
       </c>
       <c r="F197" t="n">
-        <v>3435</v>
+        <v>3437</v>
       </c>
       <c r="G197" t="n">
-        <v>0.4879184861717613</v>
+        <v>0.4879255164387547</v>
       </c>
       <c r="H197" t="inlineStr">
         <is>
@@ -16755,19 +16755,19 @@
         </is>
       </c>
       <c r="C198" t="n">
-        <v>3583</v>
+        <v>3584</v>
       </c>
       <c r="D198" t="n">
         <v>322</v>
       </c>
       <c r="E198" t="n">
-        <v>0.08986882500697739</v>
+        <v>0.08984375</v>
       </c>
       <c r="F198" t="n">
-        <v>3435</v>
+        <v>3437</v>
       </c>
       <c r="G198" t="n">
-        <v>0.09374090247452693</v>
+        <v>0.09368635437881874</v>
       </c>
       <c r="H198" t="inlineStr">
         <is>
@@ -16785,19 +16785,19 @@
         </is>
       </c>
       <c r="C199" t="n">
-        <v>3583</v>
+        <v>3584</v>
       </c>
       <c r="D199" t="n">
         <v>468</v>
       </c>
       <c r="E199" t="n">
-        <v>0.1306168015629361</v>
+        <v>0.1305803571428572</v>
       </c>
       <c r="F199" t="n">
-        <v>3435</v>
+        <v>3437</v>
       </c>
       <c r="G199" t="n">
-        <v>0.1362445414847162</v>
+        <v>0.1361652604015129</v>
       </c>
       <c r="H199" t="inlineStr">
         <is>
@@ -16848,16 +16848,16 @@
         <v>3574</v>
       </c>
       <c r="D201" t="n">
-        <v>1791</v>
+        <v>1790</v>
       </c>
       <c r="E201" t="n">
-        <v>0.5011191941801902</v>
+        <v>0.5008393956351427</v>
       </c>
       <c r="F201" t="n">
         <v>3379</v>
       </c>
       <c r="G201" t="n">
-        <v>0.5300384729209825</v>
+        <v>0.529742527374963</v>
       </c>
       <c r="H201" t="inlineStr">
         <is>
@@ -16938,16 +16938,16 @@
         <v>3574</v>
       </c>
       <c r="D204" t="n">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E204" t="n">
-        <v>0.08589815332960268</v>
+        <v>0.08617795187465026</v>
       </c>
       <c r="F204" t="n">
         <v>3379</v>
       </c>
       <c r="G204" t="n">
-        <v>0.09085528262799644</v>
+        <v>0.09115122817401598</v>
       </c>
       <c r="H204" t="inlineStr">
         <is>
@@ -16968,16 +16968,16 @@
         <v>3574</v>
       </c>
       <c r="D205" t="n">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="E205" t="n">
-        <v>0.1432568550643537</v>
+        <v>0.1435366536094012</v>
       </c>
       <c r="F205" t="n">
         <v>3379</v>
       </c>
       <c r="G205" t="n">
-        <v>0.1515241195620006</v>
+        <v>0.1518200651080201</v>
       </c>
       <c r="H205" t="inlineStr">
         <is>
@@ -17004,10 +17004,10 @@
         <v>0.01638477801268499</v>
       </c>
       <c r="F206" t="n">
-        <v>3521</v>
+        <v>3526</v>
       </c>
       <c r="G206" t="n">
-        <v>0.01760863391082079</v>
+        <v>0.01758366420873511</v>
       </c>
       <c r="H206" t="inlineStr">
         <is>
@@ -17028,16 +17028,16 @@
         <v>3784</v>
       </c>
       <c r="D207" t="n">
-        <v>1931</v>
+        <v>1941</v>
       </c>
       <c r="E207" t="n">
-        <v>0.5103065539112051</v>
+        <v>0.5129492600422833</v>
       </c>
       <c r="F207" t="n">
-        <v>3521</v>
+        <v>3526</v>
       </c>
       <c r="G207" t="n">
-        <v>0.5484237432547572</v>
+        <v>0.550482132728304</v>
       </c>
       <c r="H207" t="inlineStr">
         <is>
@@ -17058,16 +17058,16 @@
         <v>3784</v>
       </c>
       <c r="D208" t="n">
-        <v>988</v>
+        <v>992</v>
       </c>
       <c r="E208" t="n">
-        <v>0.2610993657505286</v>
+        <v>0.2621564482029599</v>
       </c>
       <c r="F208" t="n">
-        <v>3521</v>
+        <v>3526</v>
       </c>
       <c r="G208" t="n">
-        <v>0.2806021016756603</v>
+        <v>0.2813386273397618</v>
       </c>
       <c r="H208" t="inlineStr">
         <is>
@@ -17088,16 +17088,16 @@
         <v>3784</v>
       </c>
       <c r="D209" t="n">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="E209" t="n">
-        <v>0.4540169133192389</v>
+        <v>0.4542811839323467</v>
       </c>
       <c r="F209" t="n">
-        <v>3521</v>
+        <v>3526</v>
       </c>
       <c r="G209" t="n">
-        <v>0.4879295654643567</v>
+        <v>0.4875212705615428</v>
       </c>
       <c r="H209" t="inlineStr">
         <is>
@@ -17124,10 +17124,10 @@
         <v>0.08298097251585623</v>
       </c>
       <c r="F210" t="n">
-        <v>3521</v>
+        <v>3526</v>
       </c>
       <c r="G210" t="n">
-        <v>0.08917921045157626</v>
+        <v>0.0890527509926262</v>
       </c>
       <c r="H210" t="inlineStr">
         <is>
@@ -17148,16 +17148,16 @@
         <v>3784</v>
       </c>
       <c r="D211" t="n">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="E211" t="n">
-        <v>0.1400634249471459</v>
+        <v>0.1408562367864694</v>
       </c>
       <c r="F211" t="n">
-        <v>3521</v>
+        <v>3526</v>
       </c>
       <c r="G211" t="n">
-        <v>0.1505254189150809</v>
+        <v>0.1511627906976744</v>
       </c>
       <c r="H211" t="inlineStr">
         <is>
@@ -17175,19 +17175,19 @@
         </is>
       </c>
       <c r="C212" t="n">
-        <v>2717</v>
+        <v>2827</v>
       </c>
       <c r="D212" t="n">
         <v>26</v>
       </c>
       <c r="E212" t="n">
-        <v>0.009569377990430622</v>
+        <v>0.00919702865228157</v>
       </c>
       <c r="F212" t="n">
-        <v>2196</v>
+        <v>2301</v>
       </c>
       <c r="G212" t="n">
-        <v>0.01183970856102004</v>
+        <v>0.01129943502824859</v>
       </c>
       <c r="H212" t="inlineStr">
         <is>
@@ -17205,19 +17205,19 @@
         </is>
       </c>
       <c r="C213" t="n">
-        <v>2717</v>
+        <v>2827</v>
       </c>
       <c r="D213" t="n">
-        <v>1157</v>
+        <v>1217</v>
       </c>
       <c r="E213" t="n">
-        <v>0.4258373205741627</v>
+        <v>0.4304916873010258</v>
       </c>
       <c r="F213" t="n">
-        <v>2196</v>
+        <v>2301</v>
       </c>
       <c r="G213" t="n">
-        <v>0.5268670309653917</v>
+        <v>0.5289004780530204</v>
       </c>
       <c r="H213" t="inlineStr">
         <is>
@@ -17235,19 +17235,19 @@
         </is>
       </c>
       <c r="C214" t="n">
-        <v>2717</v>
+        <v>2827</v>
       </c>
       <c r="D214" t="n">
-        <v>453</v>
+        <v>475</v>
       </c>
       <c r="E214" t="n">
-        <v>0.166728008833272</v>
+        <v>0.1680226388397595</v>
       </c>
       <c r="F214" t="n">
-        <v>2196</v>
+        <v>2301</v>
       </c>
       <c r="G214" t="n">
-        <v>0.2062841530054645</v>
+        <v>0.206431986093003</v>
       </c>
       <c r="H214" t="inlineStr">
         <is>
@@ -17265,19 +17265,19 @@
         </is>
       </c>
       <c r="C215" t="n">
-        <v>2717</v>
+        <v>2827</v>
       </c>
       <c r="D215" t="n">
-        <v>1022</v>
+        <v>1065</v>
       </c>
       <c r="E215" t="n">
-        <v>0.3761501656238498</v>
+        <v>0.3767244428723028</v>
       </c>
       <c r="F215" t="n">
-        <v>2196</v>
+        <v>2301</v>
       </c>
       <c r="G215" t="n">
-        <v>0.465391621129326</v>
+        <v>0.4628422425032594</v>
       </c>
       <c r="H215" t="inlineStr">
         <is>
@@ -17295,19 +17295,19 @@
         </is>
       </c>
       <c r="C216" t="n">
-        <v>2717</v>
+        <v>2827</v>
       </c>
       <c r="D216" t="n">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="E216" t="n">
-        <v>0.05042326094957674</v>
+        <v>0.05058365758754864</v>
       </c>
       <c r="F216" t="n">
-        <v>2196</v>
+        <v>2301</v>
       </c>
       <c r="G216" t="n">
-        <v>0.06238615664845173</v>
+        <v>0.06214689265536723</v>
       </c>
       <c r="H216" t="inlineStr">
         <is>
@@ -17325,19 +17325,19 @@
         </is>
       </c>
       <c r="C217" t="n">
-        <v>2717</v>
+        <v>2827</v>
       </c>
       <c r="D217" t="n">
-        <v>299</v>
+        <v>314</v>
       </c>
       <c r="E217" t="n">
-        <v>0.1100478468899522</v>
+        <v>0.111071807569862</v>
       </c>
       <c r="F217" t="n">
-        <v>2196</v>
+        <v>2301</v>
       </c>
       <c r="G217" t="n">
-        <v>0.1361566484517304</v>
+        <v>0.1364624076488483</v>
       </c>
       <c r="H217" t="inlineStr">
         <is>

</xml_diff>